<commit_message>
data: publish 2026-10-15 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-15-182路.xlsx
+++ b/data/export/2026-10-15-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,33 +693,37 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,17 +812,17 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -820,13 +832,17 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -854,32 +870,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>76分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -887,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -911,33 +931,37 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>76.0</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -998,7 +1022,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1037,7 +1061,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
@@ -1048,7 +1072,7 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1076,32 +1100,36 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>85分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1109,7 +1137,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1133,17 +1161,17 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -1153,13 +1181,17 @@
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB6" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>4/13</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1252,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1302,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1363,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1413,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1474,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1492,7 +1524,7 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1500,22 +1532,22 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>沪A13735A</t>
+          <t>沪A68870D</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1548,12 +1580,12 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:42</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1567,7 +1599,7 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -1603,7 +1635,792 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A12050A</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>76.0</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>2/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-15 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-15-182路.xlsx
+++ b/data/export/2026-10-15-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC55"/>
+  <dimension ref="A1:AC57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>69.7</t>
+          <t>69.3</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1900,12 +1900,12 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>74.5</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2133,17 +2133,17 @@
       </c>
       <c r="AA14" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA17" s="2" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
-          <t>69.7</t>
+          <t>69.3</t>
         </is>
       </c>
       <c r="AC25" s="2" t="inlineStr">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3562,12 +3562,12 @@
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>74.5</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA27" s="2" t="inlineStr">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3795,17 +3795,17 @@
       </c>
       <c r="AA28" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="AC31" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="AC32" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
-          <t>69.7</t>
+          <t>69.3</t>
         </is>
       </c>
       <c r="AC38" s="2" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="Z39" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA39" s="2" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -5223,17 +5223,17 @@
       </c>
       <c r="AA40" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC40" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -5417,7 +5417,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="AC43" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5866,24 +5866,24 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>13:53</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>74分钟</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
-          <t>69.7</t>
+          <t>69.3</t>
         </is>
       </c>
       <c r="AC46" s="2" t="inlineStr">
@@ -5985,24 +5985,24 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:57</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>70分钟</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
@@ -6012,7 +6012,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6061,12 +6061,12 @@
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>74.5</t>
         </is>
       </c>
       <c r="AC47" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -6094,32 +6094,36 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>14:09</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>69分钟</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
           <t>07:02</t>
@@ -6127,7 +6131,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6151,17 +6155,17 @@
       </c>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X48" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z48" s="2" t="inlineStr">
@@ -6171,17 +6175,17 @@
       </c>
       <c r="AA48" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC48" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6246,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -6281,7 +6285,7 @@
       </c>
       <c r="Z49" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA49" s="2" t="inlineStr">
@@ -6296,7 +6300,7 @@
       </c>
       <c r="AC49" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6361,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -6472,7 +6476,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -6587,7 +6591,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -6702,7 +6706,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -6817,7 +6821,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -6866,12 +6870,12 @@
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>74.5</t>
         </is>
       </c>
       <c r="AC54" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -6932,7 +6936,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -6990,6 +6994,236 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr"/>
+      <c r="R56" s="2" t="inlineStr"/>
+      <c r="S56" s="2" t="inlineStr"/>
+      <c r="T56" s="2" t="inlineStr"/>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB56" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
+      <c r="AC56" s="2" t="inlineStr">
+        <is>
+          <t>3/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr"/>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr"/>
+      <c r="R57" s="2" t="inlineStr"/>
+      <c r="S57" s="2" t="inlineStr"/>
+      <c r="T57" s="2" t="inlineStr"/>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z57" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB57" s="2" t="inlineStr">
+        <is>
+          <t>76.8</t>
+        </is>
+      </c>
+      <c r="AC57" s="2" t="inlineStr">
+        <is>
+          <t>6/14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>